<commit_message>
updated figures for paper.
</commit_message>
<xml_diff>
--- a/Data/PrOACT_table.xlsx
+++ b/Data/PrOACT_table.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexandrabl/Desktop/MarEEchange/1_Paper_publi/1_SES/PrOACT/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexandrabl/Desktop/MarEEchange/1_Paper_publi/1_SES/R/prOACT_pathways/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F6868F9-88D4-6949-B3A6-D4D28529CAF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9B81123-689B-2C43-AA6F-B5262192F825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28800" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{AFCE7F91-229A-6245-B0E9-71533B67685E}"/>
   </bookViews>
@@ -516,6 +516,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{030C38E8-7FAD-C748-8EB6-79EEB55CCAB7}">
   <dimension ref="A1:Z8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A1" t="s">

</xml_diff>